<commit_message>
Add SOH report for 2026-10-20
</commit_message>
<xml_diff>
--- a/reports/SOH_19_10_2026.xlsx
+++ b/reports/SOH_19_10_2026.xlsx
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>991</v>
+        <v>971</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1145</v>
+        <v>1135</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>494</v>
+        <v>484</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>3000</v>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>2494</v>
+        <v>2493</v>
       </c>
       <c r="E110" s="3" t="n">
         <v>3500</v>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E114" s="3" t="n">
         <v>36000</v>
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>4640</v>
+        <v>4636</v>
       </c>
       <c r="E127" s="3" t="n">
         <v>2500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4601,7 +4601,7 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E149" s="3" t="n">
         <v>34890</v>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E153" s="3" t="n">
         <v>1</v>
@@ -4853,7 +4853,7 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E158" s="3" t="n">
         <v>1</v>
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>324</v>
+        <v>287</v>
       </c>
       <c r="E175" s="3" t="n">
         <v>13500</v>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E227" s="3" t="n">
         <v>1</v>
@@ -16206,7 +16206,7 @@
         </is>
       </c>
       <c r="D567" s="2" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E567" s="3" t="n">
         <v>10409</v>
@@ -16374,7 +16374,7 @@
         </is>
       </c>
       <c r="D573" s="2" t="n">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E573" s="3" t="n">
         <v>31682</v>
@@ -16458,7 +16458,7 @@
         </is>
       </c>
       <c r="D576" s="2" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E576" s="3" t="n">
         <v>10840</v>
@@ -16990,7 +16990,7 @@
         </is>
       </c>
       <c r="D595" s="2" t="n">
-        <v>332</v>
+        <v>308</v>
       </c>
       <c r="E595" s="3" t="n">
         <v>11436</v>
@@ -17775,7 +17775,7 @@
         </is>
       </c>
       <c r="D623" s="2" t="n">
-        <v>550</v>
+        <v>538</v>
       </c>
       <c r="E623" s="3" t="n">
         <v>8408</v>
@@ -17943,7 +17943,7 @@
         </is>
       </c>
       <c r="D629" s="2" t="n">
-        <v>3683</v>
+        <v>3659</v>
       </c>
       <c r="E629" s="3" t="n">
         <v>10251</v>
@@ -25728,7 +25728,7 @@
         </is>
       </c>
       <c r="D907" s="2" t="n">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E907" s="3" t="n">
         <v>14860</v>
@@ -34721,7 +34721,7 @@
         </is>
       </c>
       <c r="D1228" s="2" t="n">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E1228" s="3" t="n">
         <v>24480</v>
@@ -35001,7 +35001,7 @@
         </is>
       </c>
       <c r="D1238" s="2" t="n">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E1238" s="3" t="n">
         <v>13001</v>
@@ -35029,7 +35029,7 @@
         </is>
       </c>
       <c r="D1239" s="2" t="n">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E1239" s="3" t="n">
         <v>11269</v>
@@ -35309,7 +35309,7 @@
         </is>
       </c>
       <c r="D1249" s="2" t="n">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E1249" s="3" t="n">
         <v>14554</v>
@@ -35953,7 +35953,7 @@
         </is>
       </c>
       <c r="D1272" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E1272" s="3" t="n">
         <v>5601</v>
@@ -38697,7 +38697,7 @@
         </is>
       </c>
       <c r="D1370" s="2" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E1370" s="3" t="n">
         <v>12722</v>
@@ -40209,7 +40209,7 @@
         </is>
       </c>
       <c r="D1424" s="2" t="n">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="E1424" s="3" t="n">
         <v>3137</v>
@@ -42981,7 +42981,7 @@
         </is>
       </c>
       <c r="D1523" s="2" t="n">
-        <v>579</v>
+        <v>567</v>
       </c>
       <c r="E1523" s="3" t="n">
         <v>10729</v>
@@ -44297,7 +44297,7 @@
         </is>
       </c>
       <c r="D1570" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1570" s="3" t="n">
         <v>12610</v>
@@ -46567,7 +46567,7 @@
         </is>
       </c>
       <c r="D1651" s="2" t="n">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="E1651" s="3" t="n">
         <v>10097</v>

</xml_diff>